<commit_message>
support standard multi-sheet Amazon bulk
</commit_message>
<xml_diff>
--- a/ad-diagnostic-generator/frontend/sample-bulk.xlsx
+++ b/ad-diagnostic-generator/frontend/sample-bulk.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bulk" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sponsored Products Campaigns" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SP Search Term Report" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Portfolios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bulk'!$A$1:$R$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sponsored Products Campaigns'!$A$1:$S$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,75 +438,80 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Ad Group ID</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Portfolio ID</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Campaign Name (Informational only)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Ad Group Name (Informational only)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Portfolio Name (Informational only)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ASIN (Informational only)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Match Type</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Placement</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Product Targeting Expression</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Keyword Text</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Customer Search Term</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Orders</t>
         </is>
@@ -528,57 +535,62 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>DEMO-GROUP-1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Demo Carry-on Phrase</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Demo Group A</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Demo Portfolio</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>DEMO-SKU-A</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>B0DEMO0001</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Phrase</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>carry on luggage</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>carry on luggage</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>12500</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>315</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>264.4</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>1189.5</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>17</v>
       </c>
     </row>
@@ -600,57 +612,62 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>DEMO-GROUP-1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Demo Carry-on Phrase</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Demo Group A</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Demo Portfolio</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>DEMO-SKU-A</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>B0DEMO0001</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Phrase</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>lightweight suitcase</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>lightweight suitcase</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>6800</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>142</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>113.7</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>424</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>6</v>
       </c>
     </row>
@@ -672,57 +689,62 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>DEMO-GROUP-1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Demo Carry-on Phrase</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Demo Group A</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Demo Portfolio</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>DEMO-SKU-A</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>B0DEMO0001</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Exact</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>luggage with wheels</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>luggage with wheels</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>3100</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>61</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>58.2</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>0</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -742,34 +764,39 @@
           <t>DEMO-1001</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Demo Carry-on Phrase</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Demo Portfolio</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Placement Top</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>8900</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>228</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>205.6</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>1012</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -789,39 +816,372 @@
           <t>DEMO-1001</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Demo Carry-on Phrase</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Demo Portfolio</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Placement Product Page</t>
         </is>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>5200</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>96</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>81.3</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>302</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R6"/>
+  <autoFilter ref="A1:S6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Campaign ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Ad Group ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Campaign Name (Informational only)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ad Group Name (Informational only)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Customer Search Term</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DEMO-1001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DEMO-GROUP-1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Demo Carry-on Phrase</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Demo Group A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>carry on luggage</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>9000</v>
+      </c>
+      <c r="H2" t="n">
+        <v>250</v>
+      </c>
+      <c r="I2" t="n">
+        <v>210</v>
+      </c>
+      <c r="J2" t="n">
+        <v>900</v>
+      </c>
+      <c r="K2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DEMO-1001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DEMO-GROUP-1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Demo Carry-on Phrase</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Demo Group A</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>lightweight suitcase</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H3" t="n">
+        <v>100</v>
+      </c>
+      <c r="I3" t="n">
+        <v>80</v>
+      </c>
+      <c r="J3" t="n">
+        <v>300</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DEMO-1001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DEMO-GROUP-1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Demo Carry-on Phrase</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Demo Group A</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>luggage with wheels</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H4" t="n">
+        <v>40</v>
+      </c>
+      <c r="I4" t="n">
+        <v>35</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Portfolio ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portfolio Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Budget Amount</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Budget Currency Code</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Budget Policy</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Budget Start Date</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Budget End Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>State (Informational only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Portfolios</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Demo Portfolio</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>dateRange</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>20260601</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>20260630</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add multi-select filtering and trim output sheets
</commit_message>
<xml_diff>
--- a/ad-diagnostic-generator/frontend/sample-bulk.xlsx
+++ b/ad-diagnostic-generator/frontend/sample-bulk.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Portfolios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sponsored Products Campaigns'!$A$1:$S$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sponsored Products Campaigns'!$A$1:$S$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -852,8 +852,137 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DEMO-2002</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>DEMO-GROUP-2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Demo Checked Luggage</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Demo Group B</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Demo Portfolio</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>DEMO-SKU-B</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>B0DEMO0002</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Exact</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>checked luggage</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>4200</v>
+      </c>
+      <c r="P7" t="n">
+        <v>88</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="R7" t="n">
+        <v>356</v>
+      </c>
+      <c r="S7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bidding Adjustment</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DEMO-2002</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DEMO-PORT-1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Demo Checked Luggage</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Demo Portfolio</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Placement Top</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="P8" t="n">
+        <v>51</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="R8" t="n">
+        <v>212</v>
+      </c>
+      <c r="S8" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S6"/>
+  <autoFilter ref="A1:S8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -864,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1063,6 +1192,53 @@
       </c>
       <c r="K4" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sponsored Products</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DEMO-2002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DEMO-GROUP-2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Demo Checked Luggage</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Demo Group B</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>checked luggage</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="H5" t="n">
+        <v>72</v>
+      </c>
+      <c r="I5" t="n">
+        <v>61</v>
+      </c>
+      <c r="J5" t="n">
+        <v>305</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>